<commit_message>
Align workbook and readiness doc with run-off scope; retire Figma in favour of HTML source
</commit_message>
<xml_diff>
--- a/docs/tanachok-production-plan.xlsx
+++ b/docs/tanachok-production-plan.xlsx
@@ -7,9 +7,10 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="แผนงาน 4 เฟส" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="แผนงาน" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ประเมินความพร้อม" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ประเด็นที่ต้องตัดสินใจ" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ทบทวนฟังก์ชัน" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ประเด็นที่ต้องตัดสินใจ" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -515,7 +516,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H23"/>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -531,14 +532,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>TANACHOK (ระบบงานสลากธนโชค) — แผนทำให้พร้อมขึ้น Production</t>
+          <t>TANACHOK (ระบบงานสลากธนโชค) — แผนงานโหมดจ่ายคืน (Run-off)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>ระยะเวลาเป็นประมาณการเพื่อใช้หารือ · ต้องยืนยันกับเจ้าของระบบและหน่วยงานที่เกี่ยวข้อง</t>
+          <t>ปิดการขายแล้ว เหลือรอผู้ถือมาถอน · Phase 4 ยกเลิก · เพิ่ม Phase 5 แผนปิดระบบ · ระยะเวลาเป็นประมาณการรอยืนยัน</t>
         </is>
       </c>
     </row>
@@ -616,7 +617,11 @@
           <t>สูงมาก</t>
         </is>
       </c>
-      <c r="H5" s="4" t="inlineStr"/>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>คงไว้เต็มรูปแบบแม้ปิดการขาย</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="32" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
@@ -757,22 +762,22 @@
     <row r="10" ht="32" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>Phase 2</t>
+          <t>Phase 1</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>ทำให้ดูแลได้จริง</t>
+          <t>ปิดฟังก์ชันที่ไม่ใช้แล้ว</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>ตั้งตารางสำรองข้อมูล + ตรวจสอบไฟล์สำรองอัตโนมัติ</t>
+          <t>ปิดเมนู+ปิดสิทธิ์กลุ่ม B 7 รายการ (ขาย/ฝากเพิ่ม/ออกเลข/รางวัลงวดใหม่/รายงานขาย/พิมพ์สลาก)</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>สัปดาห์ 3-6</t>
+          <t>สัปดาห์ 1-2</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr"/>
@@ -788,7 +793,7 @@
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>ต้องได้ RPO ก่อน</t>
+          <t>ห้ามลบข้อมูล — ปิดการใช้งานเท่านั้น</t>
         </is>
       </c>
     </row>
@@ -800,12 +805,12 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>ทำให้ดูแลได้จริง</t>
+          <t>ทำให้ดูแลได้จริง (ลดขนาด)</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>ซ้อมกู้คืนจริง 1 ครั้ง จับเวลาเทียบกับ RTO ที่ตกลง</t>
+          <t>ตั้งตารางสำรองข้อมูล + ตรวจสอบไฟล์สำรองอัตโนมัติ</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
@@ -826,7 +831,7 @@
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>ต้องได้ RTO ก่อน</t>
+          <t>ต้องได้ RPO ก่อน</t>
         </is>
       </c>
     </row>
@@ -838,12 +843,12 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>ทำให้ดูแลได้จริง</t>
+          <t>ทำให้ดูแลได้จริง (ลดขนาด)</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>ติดตั้ง monitoring + alert (บริการ ดิสก์ ฐานข้อมูล ผลรัน Feed)</t>
+          <t>ซ้อมกู้คืนจริง 1 ครั้ง จับเวลาเทียบกับ RTO ที่ตกลง</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
@@ -862,7 +867,11 @@
           <t>สูง</t>
         </is>
       </c>
-      <c r="H12" s="5" t="inlineStr"/>
+      <c r="H12" s="5" t="inlineStr">
+        <is>
+          <t>RTO ยืดหยุ่นได้ในโหมดนี้</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="32" customHeight="1">
       <c r="A13" s="4" t="inlineStr">
@@ -872,12 +881,12 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>ทำให้ดูแลได้จริง</t>
+          <t>ทำให้ดูแลได้จริง (ลดขนาด)</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>ตั้ง Scheduled Task ของ Feed เป็นมาตรฐาน + แจ้งเตือนเมื่อไม่สำเร็จ</t>
+          <t>ติดตั้ง monitoring + alert เท่าที่จำเป็น (บริการ ดิสก์ ฐานข้อมูล)</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
@@ -896,7 +905,11 @@
           <t>ปานกลาง</t>
         </is>
       </c>
-      <c r="H13" s="4" t="inlineStr"/>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>ลดขอบเขตจากแผนเดิม</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="32" customHeight="1">
       <c r="A14" s="5" t="inlineStr">
@@ -906,7 +919,7 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>ทำให้ดูแลได้จริง</t>
+          <t>ทำให้ดูแลได้จริง (ลดขนาด)</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
@@ -932,7 +945,7 @@
       </c>
       <c r="H14" s="5" t="inlineStr">
         <is>
-          <t>ต้องรู้ระยะเก็บที่กำหนด</t>
+          <t>สำคัญขึ้น — เป็นหลักฐานการจ่ายคืน</t>
         </is>
       </c>
     </row>
@@ -944,7 +957,7 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>ทำให้ดูแลได้จริง</t>
+          <t>ทำให้ดูแลได้จริง (ลดขนาด)</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
@@ -973,36 +986,40 @@
     <row r="16" ht="32" customHeight="1">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>Phase 3</t>
+          <t>Phase 2</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>คุมการเปลี่ยนแปลง</t>
+          <t>ขึ้นกับการตัดสินใจ</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>นำ source code และ Stored Procedure เข้าระบบควบคุมเวอร์ชัน</t>
+          <t>งาน Feed: ตั้ง Scheduled Task + เฝ้าระวัง — หรือตัดทิ้งทั้งชุด</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>สัปดาห์ 7-12</t>
+          <t>สัปดาห์ 3-6</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr"/>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>ยังไม่เริ่ม</t>
+          <t>รอตัดสินใจ</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>สูง</t>
-        </is>
-      </c>
-      <c r="H16" s="5" t="inlineStr"/>
+          <t>ปานกลาง</t>
+        </is>
+      </c>
+      <c r="H16" s="5" t="inlineStr">
+        <is>
+          <t>รอคำตอบ C2 (ปลายทางยังต้องการไหม)</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="32" customHeight="1">
       <c r="A17" s="4" t="inlineStr">
@@ -1012,12 +1029,12 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>คุมการเปลี่ยนแปลง</t>
+          <t>คุมการเปลี่ยนแปลง (ลดเหลือเท่าที่จำเป็น)</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>ใช้ versioned migration สำหรับการแก้ฐานข้อมูล</t>
+          <t>คุมสิทธิ์การแก้ไขระบบและฐานข้อมูล</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
@@ -1046,12 +1063,12 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>คุมการเปลี่ยนแปลง</t>
+          <t>คุมการเปลี่ยนแปลง (ลดเหลือเท่าที่จำเป็น)</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>จัดทำขั้นตอน deploy มาตรฐาน + เก็บ artifact ย้อนกลับได้</t>
+          <t>นำ Stored Procedure ที่ยังใช้งานเข้าระบบควบคุมเวอร์ชัน</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
@@ -1070,7 +1087,11 @@
           <t>ปานกลาง</t>
         </is>
       </c>
-      <c r="H18" s="5" t="inlineStr"/>
+      <c r="H18" s="5" t="inlineStr">
+        <is>
+          <t>ระบบแทบไม่มีการแก้ไขแล้ว</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="32" customHeight="1">
       <c r="A19" s="4" t="inlineStr">
@@ -1080,12 +1101,12 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>คุมการเปลี่ยนแปลง</t>
+          <t>คุมการเปลี่ยนแปลง (ลดเหลือเท่าที่จำเป็น)</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>จัดทำเอกสารสถาปัตยกรรม + คู่มือปฏิบัติการรวมศูนย์</t>
+          <t>จัดทำคู่มือปฏิบัติการรวมศูนย์ + กำหนดผู้อนุมัติการเปลี่ยนแปลง</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
@@ -1109,60 +1130,64 @@
     <row r="20" ht="32" customHeight="1">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>Phase 3</t>
+          <t>Phase 4</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>คุมการเปลี่ยนแปลง</t>
+          <t>ยกระดับ/พัฒนาใหม่</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>กำหนดขั้นตอนการขอเปลี่ยนแปลง (change) และผู้อนุมัติ</t>
+          <t>ตัดออกทั้งเฟส — ไม่คุ้มที่จะรื้อระบบที่กำลังจะปิด</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>สัปดาห์ 7-12</t>
-        </is>
-      </c>
-      <c r="E20" s="5" t="inlineStr"/>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>ยังไม่เริ่ม</t>
+          <t>ยกเลิก</t>
         </is>
       </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>ปานกลาง</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H20" s="5" t="inlineStr">
         <is>
-          <t>ต้องรู้ผู้อนุมัติ</t>
+          <t>การประหยัดที่ใหญ่ที่สุดจากเงื่อนไข run-off</t>
         </is>
       </c>
     </row>
     <row r="21" ht="32" customHeight="1">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>Phase 4</t>
+          <t>Phase 5</t>
         </is>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>ยกระดับรันไทม์</t>
+          <t>แผนปิดระบบ (ใหม่)</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>ประเมินทางเลือก: ยกระดับระบบเดิม หรือ พัฒนาใหม่</t>
+          <t>กำหนดวันสิ้นสุดการรับคำขอถอน และแจ้งผู้ถือสลากล่วงหน้า</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>ประเมินหลัง Phase 3</t>
+          <t>รอกำหนด</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr"/>
@@ -1178,29 +1203,29 @@
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>ต้องมีงบประมาณ</t>
+          <t>รอคำตอบ C6</t>
         </is>
       </c>
     </row>
     <row r="22" ht="32" customHeight="1">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>Phase 4</t>
+          <t>Phase 5</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>ยกระดับรันไทม์</t>
+          <t>แผนปิดระบบ (ใหม่)</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>วิเคราะห์ผลกระทบ ค่าใช้จ่าย และระยะเวลาของแต่ละทาง</t>
+          <t>กำหนดวิธีจัดการยอดที่ไม่มีผู้มาถอนตามระเบียบ</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>ประเมินหลัง Phase 3</t>
+          <t>รอกำหนด</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr"/>
@@ -1214,27 +1239,31 @@
           <t>สูง</t>
         </is>
       </c>
-      <c r="H22" s="5" t="inlineStr"/>
+      <c r="H22" s="5" t="inlineStr">
+        <is>
+          <t>รอคำตอบ C5</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="32" customHeight="1">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>Phase 4</t>
+          <t>Phase 5</t>
         </is>
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>ยกระดับรันไทม์</t>
+          <t>แผนปิดระบบ (ใหม่)</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>เสนอเจ้าของระบบตัดสินใจเลือกแนวทาง</t>
+          <t>วางแผนเก็บข้อมูลถาวร (archive) ให้ค้นย้อนหลังได้หลังปิดระบบ</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>ประเมินหลัง Phase 3</t>
+          <t>รอกำหนด</t>
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr"/>
@@ -1249,6 +1278,74 @@
         </is>
       </c>
       <c r="H23" s="4" t="inlineStr"/>
+    </row>
+    <row r="24" ht="32" customHeight="1">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Phase 5</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>แผนปิดระบบ (ใหม่)</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>กำหนดวิธีให้บริการหากมีผู้มาติดต่อหลังปิดระบบ</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>รอกำหนด</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="inlineStr"/>
+      <c r="F24" s="5" t="inlineStr">
+        <is>
+          <t>ยังไม่เริ่ม</t>
+        </is>
+      </c>
+      <c r="G24" s="5" t="inlineStr">
+        <is>
+          <t>ปานกลาง</t>
+        </is>
+      </c>
+      <c r="H24" s="5" t="inlineStr"/>
+    </row>
+    <row r="25" ht="32" customHeight="1">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Phase 5</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>แผนปิดระบบ (ใหม่)</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>ปลดระวางเครื่องและเพิกถอนสิทธิ์เข้าถึงทั้งหมด</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>รอกำหนด</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr"/>
+      <c r="F25" s="4" t="inlineStr">
+        <is>
+          <t>ยังไม่เริ่ม</t>
+        </is>
+      </c>
+      <c r="G25" s="4" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+      <c r="H25" s="4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1280,7 +1377,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>สรุป: พร้อม 3 · บางส่วน 7 · ยังไม่มี 6 → ยังไม่ควรถือว่าพร้อม Production เต็มรูปแบบ</t>
+          <t>สรุป: พร้อม 3 · บางส่วน 7 · ยังไม่มี 6 · ประเมินก่อนทราบว่าปิดการขาย — ในโหมดจ่ายคืน ด้านความปลอดภัยยังเร่งด่วนเท่าเดิม ส่วน HA/Deploy/CI-CD ลดความสำคัญลง</t>
         </is>
       </c>
     </row>
@@ -1664,6 +1761,607 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="7" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="54" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>ทบทวนฟังก์ชันหลังปิดการขาย — คงไว้ 8 · ตัดออก 7 · รอตัดสินใจ 6</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>"ตัดออก" หมายถึงปิดการใช้งานและปิดสิทธิ์เท่านั้น — ห้ามลบข้อมูลเดิม ยังต้องเก็บเพื่อการตรวจสอบและการจ่ายคืน</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>การตัดสิน</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>ฟังก์ชัน</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>เหตุผล</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>หมายเหตุ / วิธีจัดการ</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="32" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>คงไว้</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>ค้นหาผู้ถือสลาก</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>จุดเริ่มต้นของทุกเคสเมื่อลูกค้าเดินเข้าสาขา</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr"/>
+    </row>
+    <row r="6" ht="32" customHeight="1">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>A2</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>คงไว้</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>แสดงยอดคงเหลือและสิทธิ์ที่พึงได้รับ</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>ต้องรู้ว่าจ่ายคืนเท่าไร (เงินต้น + สิทธิ์ค้างจ่าย)</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>สูตรขึ้นกับคำตอบ C3</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="32" customHeight="1">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>A3</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>คงไว้</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>บันทึกการถอน/จ่ายคืน</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>ธุรกรรมประเภทเดียวที่ยังเกิดขึ้นจริง</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr"/>
+    </row>
+    <row r="8" ht="32" customHeight="1">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>A4</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>คงไว้</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>ตรวจเงินรางวัลค้างจ่าย</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>ผู้ถือยังมีสิทธิ์รับรางวัลงวดเก่าที่ยังไม่ได้ขึ้นเงิน</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr"/>
+    </row>
+    <row r="9" ht="32" customHeight="1">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>A5</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>คงไว้</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>ประวัติธุรกรรมรายผู้ถือสลาก</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>หลักฐานการจ่ายคืน ใช้ตอบข้อโต้แย้งและการตรวจสอบ</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr"/>
+    </row>
+    <row r="10" ht="32" customHeight="1">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>A6</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>คงไว้</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>รายงานยอดคงค้างทั้งระบบ</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>ฝ่ายบัญชีต้องรู้ภาระผูกพันที่เหลือ</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr"/>
+    </row>
+    <row r="11" ht="32" customHeight="1">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>A7</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>คงไว้</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>งานปิด/ย้ายสาขา</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>สาขาทยอยปิด ต้องย้ายข้อมูลผู้ถือไปสาขาปลายทาง</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr"/>
+    </row>
+    <row r="12" ht="32" customHeight="1">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>A8</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>คงไว้</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>จัดการผู้ใช้และสิทธิ์เข้าถึง</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>ควบคุมว่าใครจ่ายเงินได้ ใครดูข้อมูลได้</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr"/>
+    </row>
+    <row r="13" ht="32" customHeight="1">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>B1</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>ตัดออก</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>ขาย/ซื้อสลากใหม่</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>ไม่เปิดขายแล้ว</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>ปิดเมนู + ปิดสิทธิ์ (ห้ามลบข้อมูล)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="32" customHeight="1">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>B2</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>ตัดออก</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>ฝากสลากเพิ่ม / ต่ออายุ</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>ไม่มีการเพิ่มยอดอีก</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>ปิดเมนู</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="32" customHeight="1">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>B3</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>ตัดออก</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>จัดสรรและออกเลขสลาก</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>ไม่มีสลากใหม่ให้ออกเลข</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>ปิดงาน + หยุด job</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="32" customHeight="1">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>B4</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>ตัดออก</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>ประมวลผลออกรางวัลงวดใหม่</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>ไม่มีงวดใหม่แล้ว</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>เก็บผลงวดเก่าไว้เพื่อ A4</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="32" customHeight="1">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>B5</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>ตัดออก</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>รายงานยอดขาย / เป้า / อันดับสาขา</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>ไม่มีการขายให้วัด</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>ปิดรายงาน</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="32" customHeight="1">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>B6</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>ตัดออก</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>ตัวเลขการขายบนหน้าภาพรวม</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>ไม่มีความหมายแล้ว</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>เปลี่ยนเป็นตัวเลขการจ่ายคืน</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="32" customHeight="1">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>B7</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>ตัดออก</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>งานพิมพ์/จัดส่งสลาก</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>ไม่มีสลากใหม่</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>ปิดงาน</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="32" customHeight="1">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+      <c r="B20" s="8" t="inlineStr">
+        <is>
+          <t>รอตัดสินใจ</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>โอนสลาก / กรณีทายาท</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>คงไว้เฉพาะมรดก หรือใช้กระบวนการเอกสารแทน</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>ถ้าคงไว้ ต้องคงหน้าจอโอน</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="32" customHeight="1">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>C2</t>
+        </is>
+      </c>
+      <c r="B21" s="8" t="inlineStr">
+        <is>
+          <t>รอตัดสินใจ</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>การส่งข้อมูลออก (SFTP Feed)</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>ปลายทางยังต้องการข้อมูลไหม / ลดความถี่ได้ไหม</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>ถ้าเลิกส่ง ตัดได้ทั้งชุด — ประหยัดมากที่สุด</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="32" customHeight="1">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>C3</t>
+        </is>
+      </c>
+      <c r="B22" s="8" t="inlineStr">
+        <is>
+          <t>รอตัดสินใจ</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>การคิดดอกเบี้ย/ผลตอบแทน</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>เดินต่อจนวันถอน หรือหยุด ณ วันที่กำหนด</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>กระทบสูตรคำนวณยอดจ่ายคืน (A2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="32" customHeight="1">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="B23" s="8" t="inlineStr">
+        <is>
+          <t>รอตัดสินใจ</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>การติดต่อผู้ถือที่ยังไม่มาถอน</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>มีแคมเปญตามตัวไหม</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>ถ้ามี ต้องเพิ่มรายงานติดตาม</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="32" customHeight="1">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>C5</t>
+        </is>
+      </c>
+      <c r="B24" s="8" t="inlineStr">
+        <is>
+          <t>รอตัดสินใจ</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>เงินที่ไม่มีผู้มาถอนตามกำหนด</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>จัดการตามระเบียบใด</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>ต้องมีขั้นตอนและรายงานรองรับ</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="32" customHeight="1">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>C6</t>
+        </is>
+      </c>
+      <c r="B25" s="8" t="inlineStr">
+        <is>
+          <t>รอตัดสินใจ</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>กำหนดวันปิดระบบ</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>มีกำหนดชัด หรือรอจนผู้ถือหมด</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>เป็นตัวกำหนดว่าจะลงทุนแค่ไหน</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1689,7 +2387,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>ใช้เป็นวาระในการประชุม — ช่องคำตอบกรอกระหว่างประชุมได้เลย</t>
+          <t>ใช้เป็นวาระในการประชุม — ช่องคำตอบกรอกระหว่างประชุมได้เลย · ประเด็นเฉพาะโหมดจ่ายคืนดูชีต "ทบทวนฟังก์ชัน" (C1-C6)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Rewrite review for confirmed platform migration to Linux/Docker/PostgreSQL
</commit_message>
<xml_diff>
--- a/docs/tanachok-production-plan.xlsx
+++ b/docs/tanachok-production-plan.xlsx
@@ -516,7 +516,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H25"/>
+  <dimension ref="A1:H31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -532,14 +532,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>TANACHOK (ระบบงานสลากธนโชค) — แผนงานโหมดจ่ายคืน (Run-off)</t>
+          <t>TANACHOK (ระบบงานสลากธนโชค) — แผนงานโหมดจ่ายคืน + ย้ายแพลตฟอร์ม</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>ปิดการขายแล้ว เหลือรอผู้ถือมาถอน · Phase 4 ยกเลิก · เพิ่ม Phase 5 แผนปิดระบบ · ระยะเวลาเป็นประมาณการรอยืนยัน</t>
+          <t>ปิดการขายแล้ว + มีมติย้ายไป Linux/Docker/PostgreSQL · หลักการ: ความปลอดภัยก่อน ย้ายทีหลัง · ระยะเวลาเป็นประมาณการรอยืนยัน</t>
         </is>
       </c>
     </row>
@@ -593,7 +593,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>ปิดความเสี่ยงเร่งด่วน</t>
+          <t>ปิดความเสี่ยงเร่งด่วน (ระบบเดิม)</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
@@ -619,7 +619,7 @@
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>คงไว้เต็มรูปแบบแม้ปิดการขาย</t>
+          <t>ทำบนระบบเดิม ไม่ต้องรอย้ายแพลตฟอร์ม</t>
         </is>
       </c>
     </row>
@@ -631,7 +631,7 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>ปิดความเสี่ยงเร่งด่วน</t>
+          <t>ปิดความเสี่ยงเร่งด่วน (ระบบเดิม)</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
@@ -655,7 +655,11 @@
           <t>สูงมาก</t>
         </is>
       </c>
-      <c r="H6" s="5" t="inlineStr"/>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>อย่ายกวิธีตั้งรหัสแบบเดิมไปแพลตฟอร์มใหม่</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="32" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
@@ -665,7 +669,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>ปิดความเสี่ยงเร่งด่วน</t>
+          <t>ปิดความเสี่ยงเร่งด่วน (ระบบเดิม)</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
@@ -699,12 +703,12 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>ปิดความเสี่ยงเร่งด่วน</t>
+          <t>ปิดความเสี่ยงเร่งด่วน (ระบบเดิม)</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>จำกัดการเข้าถึงเครือข่ายของทั้งสองเครื่องให้เหลือเท่าที่จำเป็น</t>
+          <t>จำกัดการเข้าถึงเครือข่าย (มาตรการชดเชยจนกว่าจะ cutover)</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
@@ -723,7 +727,11 @@
           <t>สูง</t>
         </is>
       </c>
-      <c r="H8" s="5" t="inlineStr"/>
+      <c r="H8" s="5" t="inlineStr">
+        <is>
+          <t>ผูกวันสิ้นสุดกับแผน cutover</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="32" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
@@ -733,12 +741,12 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>ปิดความเสี่ยงเร่งด่วน</t>
+          <t>ลดขอบเขตก่อนย้าย</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>ทบทวนว่าใครมีสิทธิ์เข้าถึงระบบอยู่บ้างในปัจจุบัน</t>
+          <t>ปิดเมนู+ปิดสิทธิ์กลุ่ม B 7 รายการ</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
@@ -757,27 +765,31 @@
           <t>สูง</t>
         </is>
       </c>
-      <c r="H9" s="4" t="inlineStr"/>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>ห้ามลบข้อมูล — และไม่ต้องยกไปแพลตฟอร์มใหม่</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="32" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>Phase 1</t>
+          <t>Phase 2</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>ปิดฟังก์ชันที่ไม่ใช้แล้ว</t>
+          <t>เตรียมจุดย้อนกลับ</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>ปิดเมนู+ปิดสิทธิ์กลุ่ม B 7 รายการ (ขาย/ฝากเพิ่ม/ออกเลข/รางวัลงวดใหม่/รายงานขาย/พิมพ์สลาก)</t>
+          <t>ตั้งตารางสำรองข้อมูล + ตรวจสอบไฟล์สำรองอัตโนมัติ</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>สัปดาห์ 1-2</t>
+          <t>สัปดาห์ 3-6</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr"/>
@@ -793,7 +805,7 @@
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>ห้ามลบข้อมูล — ปิดการใช้งานเท่านั้น</t>
+          <t>ต้องได้ RPO ก่อน</t>
         </is>
       </c>
     </row>
@@ -805,12 +817,12 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>ทำให้ดูแลได้จริง (ลดขนาด)</t>
+          <t>เตรียมจุดย้อนกลับ</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>ตั้งตารางสำรองข้อมูล + ตรวจสอบไฟล์สำรองอัตโนมัติ</t>
+          <t>ซ้อมกู้คืนจริง 1 ครั้ง</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
@@ -826,12 +838,12 @@
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>สูง</t>
+          <t>สูงมาก</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>ต้องได้ RPO ก่อน</t>
+          <t>ต้องผ่านก่อนเริ่มย้ายข้อมูลใน Phase 3</t>
         </is>
       </c>
     </row>
@@ -843,12 +855,12 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>ทำให้ดูแลได้จริง (ลดขนาด)</t>
+          <t>เตรียมจุดย้อนกลับ</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>ซ้อมกู้คืนจริง 1 ครั้ง จับเวลาเทียบกับ RTO ที่ตกลง</t>
+          <t>กำหนดนโยบายการเก็บ audit log</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
@@ -869,7 +881,7 @@
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
-          <t>RTO ยืดหยุ่นได้ในโหมดนี้</t>
+          <t>เป็นหลักฐานการจ่ายคืน</t>
         </is>
       </c>
     </row>
@@ -881,12 +893,12 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>ทำให้ดูแลได้จริง (ลดขนาด)</t>
+          <t>เตรียมจุดย้อนกลับ</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>ติดตั้ง monitoring + alert เท่าที่จำเป็น (บริการ ดิสก์ ฐานข้อมูล)</t>
+          <t>ติดตั้งการเฝ้าระวังพื้นฐาน (บริการ ดิสก์ ฐานข้อมูล)</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
@@ -905,11 +917,7 @@
           <t>ปานกลาง</t>
         </is>
       </c>
-      <c r="H13" s="4" t="inlineStr">
-        <is>
-          <t>ลดขอบเขตจากแผนเดิม</t>
-        </is>
-      </c>
+      <c r="H13" s="4" t="inlineStr"/>
     </row>
     <row r="14" ht="32" customHeight="1">
       <c r="A14" s="5" t="inlineStr">
@@ -919,12 +927,12 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>ทำให้ดูแลได้จริง (ลดขนาด)</t>
+          <t>ขึ้นกับการตัดสินใจ</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>ตรวจสอบและกำหนดนโยบายการเก็บ audit log</t>
+          <t>ตัดสินใจเรื่อง Feed — ส่งต่อ หรือยกเลิกทั้งชุด</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
@@ -935,7 +943,7 @@
       <c r="E14" s="5" t="inlineStr"/>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>ยังไม่เริ่ม</t>
+          <t>รอตัดสินใจ</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
@@ -945,29 +953,29 @@
       </c>
       <c r="H14" s="5" t="inlineStr">
         <is>
-          <t>สำคัญขึ้น — เป็นหลักฐานการจ่ายคืน</t>
+          <t>ถ้าเลิก ตัดออกจากขอบเขตการย้ายไปเลย</t>
         </is>
       </c>
     </row>
     <row r="15" ht="32" customHeight="1">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>Phase 2</t>
+          <t>Phase 3</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>ทำให้ดูแลได้จริง (ลดขนาด)</t>
+          <t>เตรียมย้ายแพลตฟอร์ม</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>ปิดงานย้ายระบบที่ยังค้าง</t>
+          <t>ยืนยันขอบเขตที่จะย้าย = เฉพาะ 8 ฟังก์ชันกลุ่ม A</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>สัปดาห์ 3-6</t>
+          <t>สัปดาห์ 7-16</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr"/>
@@ -978,7 +986,7 @@
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>ปานกลาง</t>
+          <t>สูงมาก</t>
         </is>
       </c>
       <c r="H15" s="4" t="inlineStr"/>
@@ -986,38 +994,38 @@
     <row r="16" ht="32" customHeight="1">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>Phase 2</t>
+          <t>Phase 3</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>ขึ้นกับการตัดสินใจ</t>
+          <t>เตรียมย้ายแพลตฟอร์ม</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>งาน Feed: ตั้ง Scheduled Task + เฝ้าระวัง — หรือตัดทิ้งทั้งชุด</t>
+          <t>เขียน Stored Procedure ที่ยังใช้จริงใหม่บน PostgreSQL</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>สัปดาห์ 3-6</t>
+          <t>สัปดาห์ 7-16</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr"/>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>รอตัดสินใจ</t>
+          <t>ยังไม่เริ่ม</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>ปานกลาง</t>
+          <t>สูงมาก</t>
         </is>
       </c>
       <c r="H16" s="5" t="inlineStr">
         <is>
-          <t>รอคำตอบ C2 (ปลายทางยังต้องการไหม)</t>
+          <t>T-SQL ย้ายตรง ๆ ไม่ได้</t>
         </is>
       </c>
     </row>
@@ -1029,17 +1037,17 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>คุมการเปลี่ยนแปลง (ลดเหลือเท่าที่จำเป็น)</t>
+          <t>เตรียมย้ายแพลตฟอร์ม</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>คุมสิทธิ์การแก้ไขระบบและฐานข้อมูล</t>
+          <t>ย้ายโครงสร้างและข้อมูลจริง + กำหนด encoding ภาษาไทย/ชนิดข้อมูลจำนวนเงิน</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>สัปดาห์ 7-12</t>
+          <t>สัปดาห์ 7-16</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr"/>
@@ -1050,10 +1058,14 @@
       </c>
       <c r="G17" s="4" t="inlineStr">
         <is>
-          <t>สูง</t>
-        </is>
-      </c>
-      <c r="H17" s="4" t="inlineStr"/>
+          <t>สูงมาก</t>
+        </is>
+      </c>
+      <c r="H17" s="4" t="inlineStr">
+        <is>
+          <t>UTF-8 · เลขทศนิยมห้ามปัดเศษ</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="32" customHeight="1">
       <c r="A18" s="5" t="inlineStr">
@@ -1063,17 +1075,17 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>คุมการเปลี่ยนแปลง (ลดเหลือเท่าที่จำเป็น)</t>
+          <t>เตรียมย้ายแพลตฟอร์ม</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>นำ Stored Procedure ที่ยังใช้งานเข้าระบบควบคุมเวอร์ชัน</t>
+          <t>กระทบยอด (reconciliation) ทุกบัญชีทุกบาท เทียบระบบเก่า-ใหม่</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>สัปดาห์ 7-12</t>
+          <t>สัปดาห์ 7-16</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr"/>
@@ -1084,12 +1096,12 @@
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>ปานกลาง</t>
+          <t>สูงมาก</t>
         </is>
       </c>
       <c r="H18" s="5" t="inlineStr">
         <is>
-          <t>ระบบแทบไม่มีการแก้ไขแล้ว</t>
+          <t>หัวใจของโครงการ</t>
         </is>
       </c>
     </row>
@@ -1101,17 +1113,17 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>คุมการเปลี่ยนแปลง (ลดเหลือเท่าที่จำเป็น)</t>
+          <t>เตรียมย้ายแพลตฟอร์ม</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>จัดทำคู่มือปฏิบัติการรวมศูนย์ + กำหนดผู้อนุมัติการเปลี่ยนแปลง</t>
+          <t>ยกประวัติธุรกรรมเดิมไปด้วย + ทดสอบค้นย้อนหลัง</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>สัปดาห์ 7-12</t>
+          <t>สัปดาห์ 7-16</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr"/>
@@ -1122,72 +1134,72 @@
       </c>
       <c r="G19" s="4" t="inlineStr">
         <is>
-          <t>ปานกลาง</t>
-        </is>
-      </c>
-      <c r="H19" s="4" t="inlineStr"/>
+          <t>สูง</t>
+        </is>
+      </c>
+      <c r="H19" s="4" t="inlineStr">
+        <is>
+          <t>ร่องรอยต้องไม่ขาดตอน</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="32" customHeight="1">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>Phase 4</t>
+          <t>Phase 3</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>ยกระดับ/พัฒนาใหม่</t>
+          <t>เตรียมย้ายแพลตฟอร์ม</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>ตัดออกทั้งเฟส — ไม่คุ้มที่จะรื้อระบบที่กำลังจะปิด</t>
+          <t>ย้ายงาน Feed ไปสคริปต์ฉบับ Linux + ทดสอบตามชุด TC เดิม</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E20" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+          <t>สัปดาห์ 7-16</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr"/>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>ยกเลิก</t>
+          <t>ยังไม่เริ่ม</t>
         </is>
       </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>ปานกลาง</t>
         </is>
       </c>
       <c r="H20" s="5" t="inlineStr">
         <is>
-          <t>การประหยัดที่ใหญ่ที่สุดจากเงื่อนไข run-off</t>
+          <t>ถ้ายังต้องส่ง (ดูชีตทบทวนฟังก์ชัน C2)</t>
         </is>
       </c>
     </row>
     <row r="21" ht="32" customHeight="1">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>Phase 5</t>
+          <t>Phase 3</t>
         </is>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>แผนปิดระบบ (ใหม่)</t>
+          <t>เตรียมย้ายแพลตฟอร์ม</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>กำหนดวันสิ้นสุดการรับคำขอถอน และแจ้งผู้ถือสลากล่วงหน้า</t>
+          <t>นำโค้ดและสคริปต์ย้ายข้อมูลเข้าระบบควบคุมเวอร์ชัน + คู่มือปฏิบัติการ</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>รอกำหนด</t>
+          <t>สัปดาห์ 7-16</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr"/>
@@ -1201,31 +1213,27 @@
           <t>สูง</t>
         </is>
       </c>
-      <c r="H21" s="4" t="inlineStr">
-        <is>
-          <t>รอคำตอบ C6</t>
-        </is>
-      </c>
+      <c r="H21" s="4" t="inlineStr"/>
     </row>
     <row r="22" ht="32" customHeight="1">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>Phase 5</t>
+          <t>Phase 4</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>แผนปิดระบบ (ใหม่)</t>
+          <t>รันคู่ขนานและ Cutover</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>กำหนดวิธีจัดการยอดที่ไม่มีผู้มาถอนตามระเบียบ</t>
+          <t>รันคู่ขนานอย่างน้อย 1 รอบเต็ม เทียบผลระบบเก่า-ใหม่</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>รอกำหนด</t>
+          <t>หลัง Phase 3</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr"/>
@@ -1236,34 +1244,30 @@
       </c>
       <c r="G22" s="5" t="inlineStr">
         <is>
-          <t>สูง</t>
-        </is>
-      </c>
-      <c r="H22" s="5" t="inlineStr">
-        <is>
-          <t>รอคำตอบ C5</t>
-        </is>
-      </c>
+          <t>สูงมาก</t>
+        </is>
+      </c>
+      <c r="H22" s="5" t="inlineStr"/>
     </row>
     <row r="23" ht="32" customHeight="1">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>Phase 5</t>
+          <t>Phase 4</t>
         </is>
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>แผนปิดระบบ (ใหม่)</t>
+          <t>รันคู่ขนานและ Cutover</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>วางแผนเก็บข้อมูลถาวร (archive) ให้ค้นย้อนหลังได้หลังปิดระบบ</t>
+          <t>ให้ผู้ใช้จริงทดสอบการจ่ายคืนบนระบบใหม่ (UAT)</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>รอกำหนด</t>
+          <t>หลัง Phase 3</t>
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr"/>
@@ -1282,22 +1286,22 @@
     <row r="24" ht="32" customHeight="1">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>Phase 5</t>
+          <t>Phase 4</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>แผนปิดระบบ (ใหม่)</t>
+          <t>รันคู่ขนานและ Cutover</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>กำหนดวิธีให้บริการหากมีผู้มาติดต่อหลังปิดระบบ</t>
+          <t>กำหนดเกณฑ์ผ่าน/ไม่ผ่าน + แผนย้อนกลับหากยอดไม่ตรง</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>รอกำหนด</t>
+          <t>หลัง Phase 3</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr"/>
@@ -1308,7 +1312,7 @@
       </c>
       <c r="G24" s="5" t="inlineStr">
         <is>
-          <t>ปานกลาง</t>
+          <t>สูงมาก</t>
         </is>
       </c>
       <c r="H24" s="5" t="inlineStr"/>
@@ -1316,22 +1320,22 @@
     <row r="25" ht="32" customHeight="1">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>Phase 5</t>
+          <t>Phase 4</t>
         </is>
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>แผนปิดระบบ (ใหม่)</t>
+          <t>รันคู่ขนานและ Cutover</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>ปลดระวางเครื่องและเพิกถอนสิทธิ์เข้าถึงทั้งหมด</t>
+          <t>เลือกช่วง cutover ที่มีผู้มาถอนน้อย + แจ้งสาขาล่วงหน้า</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>รอกำหนด</t>
+          <t>หลัง Phase 3</t>
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr"/>
@@ -1346,6 +1350,214 @@
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr"/>
+    </row>
+    <row r="26" ht="32" customHeight="1">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Phase 4</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>รันคู่ขนานและ Cutover</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>cutover + เฝ้าระวังใกล้ชิด · ปลดระวางเครื่อง Windows เดิมเมื่อระบบใหม่นิ่ง</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>หลัง Phase 3</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr"/>
+      <c r="F26" s="5" t="inlineStr">
+        <is>
+          <t>ยังไม่เริ่ม</t>
+        </is>
+      </c>
+      <c r="G26" s="5" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+      <c r="H26" s="5" t="inlineStr"/>
+    </row>
+    <row r="27" ht="32" customHeight="1">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Phase 5</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>แผนปิดระบบ</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>กำหนดวันสิ้นสุดการรับคำขอถอน และแจ้งผู้ถือสลากล่วงหน้า</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>รอกำหนด</t>
+        </is>
+      </c>
+      <c r="E27" s="4" t="inlineStr"/>
+      <c r="F27" s="4" t="inlineStr">
+        <is>
+          <t>ยังไม่เริ่ม</t>
+        </is>
+      </c>
+      <c r="G27" s="4" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+      <c r="H27" s="4" t="inlineStr">
+        <is>
+          <t>ตัวกำหนดว่าจะย้ายแพลตฟอร์มหรือไม่</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="32" customHeight="1">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Phase 5</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>แผนปิดระบบ</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>กำหนดวิธีจัดการยอดที่ไม่มีผู้มาถอนตามระเบียบ</t>
+        </is>
+      </c>
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>รอกำหนด</t>
+        </is>
+      </c>
+      <c r="E28" s="5" t="inlineStr"/>
+      <c r="F28" s="5" t="inlineStr">
+        <is>
+          <t>ยังไม่เริ่ม</t>
+        </is>
+      </c>
+      <c r="G28" s="5" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+      <c r="H28" s="5" t="inlineStr"/>
+    </row>
+    <row r="29" ht="32" customHeight="1">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Phase 5</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>แผนปิดระบบ</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>วางแผนเก็บข้อมูลถาวร (archive) ให้ค้นย้อนหลังได้</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>รอกำหนด</t>
+        </is>
+      </c>
+      <c r="E29" s="4" t="inlineStr"/>
+      <c r="F29" s="4" t="inlineStr">
+        <is>
+          <t>ยังไม่เริ่ม</t>
+        </is>
+      </c>
+      <c r="G29" s="4" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+      <c r="H29" s="4" t="inlineStr"/>
+    </row>
+    <row r="30" ht="32" customHeight="1">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Phase 5</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>แผนปิดระบบ</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>กำหนดวิธีให้บริการหากมีผู้มาติดต่อหลังปิดระบบ</t>
+        </is>
+      </c>
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>รอกำหนด</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="inlineStr"/>
+      <c r="F30" s="5" t="inlineStr">
+        <is>
+          <t>ยังไม่เริ่ม</t>
+        </is>
+      </c>
+      <c r="G30" s="5" t="inlineStr">
+        <is>
+          <t>ปานกลาง</t>
+        </is>
+      </c>
+      <c r="H30" s="5" t="inlineStr"/>
+    </row>
+    <row r="31" ht="32" customHeight="1">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Phase 5</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>แผนปิดระบบ</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="inlineStr">
+        <is>
+          <t>ปลดระวางระบบและเพิกถอนสิทธิ์เข้าถึงทั้งหมด</t>
+        </is>
+      </c>
+      <c r="D31" s="4" t="inlineStr">
+        <is>
+          <t>รอกำหนด</t>
+        </is>
+      </c>
+      <c r="E31" s="4" t="inlineStr"/>
+      <c r="F31" s="4" t="inlineStr">
+        <is>
+          <t>ยังไม่เริ่ม</t>
+        </is>
+      </c>
+      <c r="G31" s="4" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+      <c r="H31" s="4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1377,7 +1589,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>สรุป: พร้อม 3 · บางส่วน 7 · ยังไม่มี 6 · ประเมินก่อนทราบว่าปิดการขาย — ในโหมดจ่ายคืน ด้านความปลอดภัยยังเร่งด่วนเท่าเดิม ส่วน HA/Deploy/CI-CD ลดความสำคัญลง</t>
+          <t>ประเมินระบบเดิมที่ยังใช้งานอยู่ · พร้อม 3 · บางส่วน 7 · ยังไม่มี 6 — รันไทม์/App Server แก้ด้วยการย้ายแพลตฟอร์ม ส่วนรหัสผ่าน/สำรองข้อมูล/audit log ต้องทำทันทีบนระบบเดิม</t>
         </is>
       </c>
     </row>
@@ -1465,7 +1677,7 @@
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>รันไทม์หมดการสนับสนุน ไม่มี security patch</t>
+          <t>หมดการสนับสนุน — แก้ด้วยการย้ายแพลตฟอร์ม ระหว่างรอใช้มาตรการชดเชย</t>
         </is>
       </c>
     </row>
@@ -1487,7 +1699,7 @@
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>ตัวให้บริการเว็บหมดการสนับสนุน ไม่มีผู้ผลิตดูแล</t>
+          <t>หมดการสนับสนุน — แก้ด้วยการย้ายแพลตฟอร์ม</t>
         </is>
       </c>
     </row>
@@ -1663,7 +1875,7 @@
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>Stored Procedure แก้ตรงเครื่อง ไม่มี versioned migration</t>
+          <t>ต้องคุมเวอร์ชันตอนเขียน SP ใหม่บน PostgreSQL</t>
         </is>
       </c>
     </row>
@@ -2367,7 +2579,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2426,16 +2638,20 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>ระบบใช้งานช่วงเวลาใด และช่วงไหนห้ามหยุด</t>
+          <t>ย้ายแพลตฟอร์มคุ้มกับความเสี่ยงหรือไม่ เมื่อระบบกำลังจะปิด</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>กำหนด change window และแผน DR</t>
+          <t>ถ้าวันปิดใกล้พอ การคงระบบเดิมพร้อมมาตรการชดเชยอาจเสี่ยงน้อยกว่า</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr"/>
-      <c r="E5" s="4" t="inlineStr"/>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>บล็อก Phase 3-4 ทั้งหมด</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="32" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
@@ -2445,18 +2661,18 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>ยอมให้ระบบหยุดได้นานเท่าใด (RTO)</t>
+          <t>เกณฑ์การกระทบยอดที่ยอมรับได้คืออะไร</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>ออกแบบเครื่องสำรอง/ขั้นตอนกู้คืน</t>
+          <t>ต้องตรงทุกบาท หรือมีเกณฑ์ผ่อนผัน — ใช้เป็นเกณฑ์ cutover</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr"/>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>บล็อก Phase 2</t>
+          <t>บล็อก Phase 4</t>
         </is>
       </c>
     </row>
@@ -2468,18 +2684,18 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>ยอมให้ข้อมูลหายได้ถึงจุดใด (RPO)</t>
+          <t>ยืนยันย้ายเฉพาะ 8 ฟังก์ชันกลุ่ม A ได้หรือไม่</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>กำหนดความถี่การสำรองข้อมูล</t>
+          <t>ลดงานเขียน SP ใหม่และงานทดสอบลงมาก</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr"/>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>บล็อก Phase 2</t>
+          <t>กำหนดขอบเขต Phase 3</t>
         </is>
       </c>
     </row>
@@ -2491,12 +2707,12 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>ต้องเก็บข้อมูล/log ย้อนหลังกี่ปี</t>
+          <t>ระบบใช้งานช่วงเวลาใด และช่วงไหนห้ามหยุด</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>กำหนดพื้นที่จัดเก็บและนโยบาย</t>
+          <t>กำหนด change window และช่วง cutover</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr"/>
@@ -2510,16 +2726,20 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>ผู้ใช้งานกี่คน สาขา/ส่วนกลาง</t>
+          <t>ยอมให้ระบบหยุดได้นานเท่าใด (RTO)</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>ประเมินขนาดเครื่องและสิทธิ์</t>
+          <t>ออกแบบเครื่องสำรอง/ขั้นตอนกู้คืน</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr"/>
-      <c r="E9" s="4" t="inlineStr"/>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>บล็อก Phase 2</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="32" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
@@ -2529,16 +2749,20 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>ระบบปลายทางของ SFTP Feed คือระบบใด ใครดูแล</t>
+          <t>ยอมให้ข้อมูลหายได้ถึงจุดใด (RPO)</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>กำหนดผู้ประสานงานและ SLA ของ Feed</t>
+          <t>กำหนดความถี่การสำรองข้อมูล</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr"/>
-      <c r="E10" s="5" t="inlineStr"/>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>บล็อก Phase 2</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="32" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
@@ -2548,12 +2772,12 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>ใครคือผู้อนุมัติการเปลี่ยนแปลงระบบ</t>
+          <t>ต้องเก็บข้อมูล/log ย้อนหลังกี่ปี</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>ตั้งขั้นตอน change management</t>
+          <t>กำหนดพื้นที่จัดเก็บและนโยบาย</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr"/>
@@ -2567,12 +2791,12 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>ใครดูแลระบบหลัง go-live และช่วงเวลาใด</t>
+          <t>ผู้ใช้งานกี่คน สาขา/ส่วนกลาง</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>กำหนดรูปแบบการสนับสนุน</t>
+          <t>ประเมินขนาดเครื่องและสิทธิ์</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr"/>
@@ -2586,20 +2810,16 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>งบประมาณ/กรอบเวลาสำหรับ Phase 4</t>
+          <t>ระบบปลายทางของ SFTP Feed คือระบบใด ใครดูแล</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>เลือกระหว่างยกระดับกับพัฒนาใหม่</t>
+          <t>กำหนดผู้ประสานงานและ SLA ของ Feed</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr"/>
-      <c r="E13" s="4" t="inlineStr">
-        <is>
-          <t>บล็อก Phase 4</t>
-        </is>
-      </c>
+      <c r="E13" s="4" t="inlineStr"/>
     </row>
     <row r="14" ht="32" customHeight="1">
       <c r="A14" s="5" t="inlineStr">
@@ -2609,16 +2829,77 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>มีข้อกำหนดจากผู้กำกับ/ผู้ตรวจสอบเพิ่มหรือไม่</t>
+          <t>ใครคือผู้อนุมัติการเปลี่ยนแปลงระบบ</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>ปรับแผนให้สอดคล้อง</t>
+          <t>ตั้งขั้นตอน change management</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr"/>
       <c r="E14" s="5" t="inlineStr"/>
+    </row>
+    <row r="15" ht="32" customHeight="1">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>ใครดูแลระบบหลัง go-live และช่วงเวลาใด</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>กำหนดรูปแบบการสนับสนุน</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr"/>
+      <c r="E15" s="4" t="inlineStr"/>
+    </row>
+    <row r="16" ht="32" customHeight="1">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>งบประมาณ/กรอบเวลาสำหรับการย้ายแพลตฟอร์ม</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>กำหนดว่าทำได้จริงในกรอบเวลาไหน</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr"/>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>บล็อก Phase 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="32" customHeight="1">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>มีข้อกำหนดจากผู้กำกับ/ผู้ตรวจสอบเพิ่มหรือไม่</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>ปรับแผนให้สอดคล้อง</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr"/>
+      <c r="E17" s="4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add CI/CD section based on Linkage Center standard
TANACHOK จะใช้กระบวนการ CI/CD เดียวกับ Linkage Center 2 ซึ่งผ่านมาตรฐาน
ธนาคารมาแล้ว จึงเพิ่มเนื้อหาเข้าเอกสารรีวิว หน้าเว็บ สไลด์ และแผนงาน:

- ส่วนที่ 8 ใหม่: เครื่องมือ, เอกสารขอใช้ 4 ฉบับ, โครงสร้าง branch,
  pipeline 4 ตัว (SIT/UAT/SEC/PROD), Deploy Checklist และบทเรียนจาก LK
- ข้อจำกัดสำคัญ: Jenkins ธนาคารไม่ต่ออินเทอร์เน็ต ต้องทำ Base Image ส่งก่อน
- เพิ่มรายการตรวจ CI/CD เข้า Phase 3 และ Phase 4 (รวม vite build -> nginx)
- เพิ่ม 2 สไลด์ และเพิ่มแถวงาน CI/CD ในชีตแผนงาน

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012L2ocaTqFvwuT3bf5E4GuQ
</commit_message>
<xml_diff>
--- a/docs/tanachok-production-plan.xlsx
+++ b/docs/tanachok-production-plan.xlsx
@@ -516,7 +516,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H31"/>
+  <dimension ref="A1:H37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1218,22 +1218,22 @@
     <row r="22" ht="32" customHeight="1">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>Phase 4</t>
+          <t>Phase 3</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>รันคู่ขนานและ Cutover</t>
+          <t>CI/CD (ตามมาตรฐาน Linkage Center)</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>รันคู่ขนานอย่างน้อย 1 รอบเต็ม เทียบผลระบบเก่า-ใหม่</t>
+          <t>ยื่นเอกสารขอใช้ CI/CD กับทีม QA 4 ฉบับ (แบบฟอร์ม CICD · Jenkinsfile · Firewall Policy · คู่มือ GitLab)</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>หลัง Phase 3</t>
+          <t>สัปดาห์ 7-16</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr"/>
@@ -1244,30 +1244,34 @@
       </c>
       <c r="G22" s="5" t="inlineStr">
         <is>
-          <t>สูงมาก</t>
-        </is>
-      </c>
-      <c r="H22" s="5" t="inlineStr"/>
+          <t>สูง</t>
+        </is>
+      </c>
+      <c r="H22" s="5" t="inlineStr">
+        <is>
+          <t>ยื่นแต่เนิ่น ๆ — งานเอกสาร+ขอเปิด firewall ใช้เวลาเป็นสัปดาห์ถึงเดือน</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="32" customHeight="1">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>Phase 4</t>
+          <t>Phase 3</t>
         </is>
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>รันคู่ขนานและ Cutover</t>
+          <t>CI/CD (ตามมาตรฐาน Linkage Center)</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>ให้ผู้ใช้จริงทดสอบการจ่ายคืนบนระบบใหม่ (UAT)</t>
+          <t>จัดทำ Base Image นำส่งธนาคาร (runtime API · Node.js สำหรับ build หน้าเว็บ · เครื่องมือ migration + PostgreSQL client)</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>หลัง Phase 3</t>
+          <t>สัปดาห์ 7-16</t>
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr"/>
@@ -1278,30 +1282,34 @@
       </c>
       <c r="G23" s="4" t="inlineStr">
         <is>
-          <t>สูง</t>
-        </is>
-      </c>
-      <c r="H23" s="4" t="inlineStr"/>
+          <t>สูงมาก</t>
+        </is>
+      </c>
+      <c r="H23" s="4" t="inlineStr">
+        <is>
+          <t>Jenkins ของธนาคารไม่ต่ออินเทอร์เน็ต — ต้องมี dependency ครบในภาพ</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="32" customHeight="1">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>Phase 4</t>
+          <t>Phase 3</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>รันคู่ขนานและ Cutover</t>
+          <t>CI/CD (ตามมาตรฐาน Linkage Center)</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>กำหนดเกณฑ์ผ่าน/ไม่ผ่าน + แผนย้อนกลับหากยอดไม่ตรง</t>
+          <t>ตั้ง repository ใน GitLab ธนาคาร + branch main/dev + กำหนดผู้อนุมัติ Merge Request ฝั่งธนาคาร</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>หลัง Phase 3</t>
+          <t>สัปดาห์ 7-16</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr"/>
@@ -1312,30 +1320,34 @@
       </c>
       <c r="G24" s="5" t="inlineStr">
         <is>
-          <t>สูงมาก</t>
-        </is>
-      </c>
-      <c r="H24" s="5" t="inlineStr"/>
+          <t>สูง</t>
+        </is>
+      </c>
+      <c r="H24" s="5" t="inlineStr">
+        <is>
+          <t>ติด Tag version (vx.x.xx) ได้ที่ main เท่านั้น</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="32" customHeight="1">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>Phase 4</t>
+          <t>Phase 3</t>
         </is>
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>รันคู่ขนานและ Cutover</t>
+          <t>CI/CD (ตามมาตรฐาน Linkage Center)</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>เลือกช่วง cutover ที่มีผู้มาถอนน้อย + แจ้งสาขาล่วงหน้า</t>
+          <t>ทำ vite build เป็นขั้นตอนใน pipeline แล้วเสิร์ฟผ่าน nginx</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>หลัง Phase 3</t>
+          <t>สัปดาห์ 7-16</t>
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr"/>
@@ -1346,30 +1358,34 @@
       </c>
       <c r="G25" s="4" t="inlineStr">
         <is>
-          <t>สูง</t>
-        </is>
-      </c>
-      <c r="H25" s="4" t="inlineStr"/>
+          <t>ปานกลาง</t>
+        </is>
+      </c>
+      <c r="H25" s="4" t="inlineStr">
+        <is>
+          <t>เลิกใช้ Vite dev server ทุก env ที่สูงกว่า dev</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="32" customHeight="1">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>Phase 4</t>
+          <t>Phase 3</t>
         </is>
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>รันคู่ขนานและ Cutover</t>
+          <t>CI/CD (ตามมาตรฐาน Linkage Center)</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>cutover + เฝ้าระวังใกล้ชิด · ปลดระวางเครื่อง Windows เดิมเมื่อระบบใหม่นิ่ง</t>
+          <t>ฝัง Tag version ลงใน image + ทำหน้าจอแสดง version</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>หลัง Phase 3</t>
+          <t>สัปดาห์ 7-16</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr"/>
@@ -1380,30 +1396,34 @@
       </c>
       <c r="G26" s="5" t="inlineStr">
         <is>
-          <t>สูง</t>
-        </is>
-      </c>
-      <c r="H26" s="5" t="inlineStr"/>
+          <t>ปานกลาง</t>
+        </is>
+      </c>
+      <c r="H26" s="5" t="inlineStr">
+        <is>
+          <t>ธนาคารกำหนดให้ตรวจสอบ version ที่ deploy ได้จากหน้าจอ</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="32" customHeight="1">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>Phase 5</t>
+          <t>Phase 4</t>
         </is>
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>แผนปิดระบบ</t>
+          <t>รันคู่ขนานและ Cutover</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>กำหนดวันสิ้นสุดการรับคำขอถอน และแจ้งผู้ถือสลากล่วงหน้า</t>
+          <t>รันคู่ขนานอย่างน้อย 1 รอบเต็ม เทียบผลระบบเก่า-ใหม่</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>รอกำหนด</t>
+          <t>หลัง Phase 3</t>
         </is>
       </c>
       <c r="E27" s="4" t="inlineStr"/>
@@ -1414,34 +1434,30 @@
       </c>
       <c r="G27" s="4" t="inlineStr">
         <is>
-          <t>สูง</t>
-        </is>
-      </c>
-      <c r="H27" s="4" t="inlineStr">
-        <is>
-          <t>ตัวกำหนดว่าจะย้ายแพลตฟอร์มหรือไม่</t>
-        </is>
-      </c>
+          <t>สูงมาก</t>
+        </is>
+      </c>
+      <c r="H27" s="4" t="inlineStr"/>
     </row>
     <row r="28" ht="32" customHeight="1">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>Phase 5</t>
+          <t>Phase 4</t>
         </is>
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>แผนปิดระบบ</t>
+          <t>รันคู่ขนานและ Cutover</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>กำหนดวิธีจัดการยอดที่ไม่มีผู้มาถอนตามระเบียบ</t>
+          <t>ให้ผู้ใช้จริงทดสอบการจ่ายคืนบนระบบใหม่ (UAT)</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>รอกำหนด</t>
+          <t>หลัง Phase 3</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr"/>
@@ -1460,22 +1476,22 @@
     <row r="29" ht="32" customHeight="1">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>Phase 5</t>
+          <t>Phase 4</t>
         </is>
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>แผนปิดระบบ</t>
+          <t>รันคู่ขนานและ Cutover</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>วางแผนเก็บข้อมูลถาวร (archive) ให้ค้นย้อนหลังได้</t>
+          <t>กำหนดเกณฑ์ผ่าน/ไม่ผ่าน + แผนย้อนกลับหากยอดไม่ตรง</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>รอกำหนด</t>
+          <t>หลัง Phase 3</t>
         </is>
       </c>
       <c r="E29" s="4" t="inlineStr"/>
@@ -1486,7 +1502,7 @@
       </c>
       <c r="G29" s="4" t="inlineStr">
         <is>
-          <t>สูง</t>
+          <t>สูงมาก</t>
         </is>
       </c>
       <c r="H29" s="4" t="inlineStr"/>
@@ -1494,22 +1510,22 @@
     <row r="30" ht="32" customHeight="1">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>Phase 5</t>
+          <t>Phase 4</t>
         </is>
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>แผนปิดระบบ</t>
+          <t>รันคู่ขนานและ Cutover</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>กำหนดวิธีให้บริการหากมีผู้มาติดต่อหลังปิดระบบ</t>
+          <t>ปรับ Deploy Checklist ของ LK เป็นฉบับธนโชค (mysqldump -&gt; pg_dump) + เพิ่มข้อตรวจยอดคงเหลือลูกค้าหลัง deploy</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>รอกำหนด</t>
+          <t>หลัง Phase 3</t>
         </is>
       </c>
       <c r="E30" s="5" t="inlineStr"/>
@@ -1520,30 +1536,34 @@
       </c>
       <c r="G30" s="5" t="inlineStr">
         <is>
-          <t>ปานกลาง</t>
-        </is>
-      </c>
-      <c r="H30" s="5" t="inlineStr"/>
+          <t>สูงมาก</t>
+        </is>
+      </c>
+      <c r="H30" s="5" t="inlineStr">
+        <is>
+          <t>LK ไม่มีข้อตรวจยอดเงิน เพราะไม่ได้ถือเงินลูกค้า · rollback ห้ามใช้ --force-recreate</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="32" customHeight="1">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>Phase 5</t>
+          <t>Phase 4</t>
         </is>
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>แผนปิดระบบ</t>
+          <t>รันคู่ขนานและ Cutover</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>ปลดระวางระบบและเพิกถอนสิทธิ์เข้าถึงทั้งหมด</t>
+          <t>เลือกช่วง cutover ที่มีผู้มาถอนน้อย + แจ้งสาขาล่วงหน้า</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>รอกำหนด</t>
+          <t>หลัง Phase 3</t>
         </is>
       </c>
       <c r="E31" s="4" t="inlineStr"/>
@@ -1558,6 +1578,214 @@
         </is>
       </c>
       <c r="H31" s="4" t="inlineStr"/>
+    </row>
+    <row r="32" ht="32" customHeight="1">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>Phase 4</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>รันคู่ขนานและ Cutover</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>cutover + เฝ้าระวังใกล้ชิด · ปลดระวางเครื่อง Windows เดิมเมื่อระบบใหม่นิ่ง</t>
+        </is>
+      </c>
+      <c r="D32" s="5" t="inlineStr">
+        <is>
+          <t>หลัง Phase 3</t>
+        </is>
+      </c>
+      <c r="E32" s="5" t="inlineStr"/>
+      <c r="F32" s="5" t="inlineStr">
+        <is>
+          <t>ยังไม่เริ่ม</t>
+        </is>
+      </c>
+      <c r="G32" s="5" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+      <c r="H32" s="5" t="inlineStr"/>
+    </row>
+    <row r="33" ht="32" customHeight="1">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Phase 5</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>แผนปิดระบบ</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
+          <t>กำหนดวันสิ้นสุดการรับคำขอถอน และแจ้งผู้ถือสลากล่วงหน้า</t>
+        </is>
+      </c>
+      <c r="D33" s="4" t="inlineStr">
+        <is>
+          <t>รอกำหนด</t>
+        </is>
+      </c>
+      <c r="E33" s="4" t="inlineStr"/>
+      <c r="F33" s="4" t="inlineStr">
+        <is>
+          <t>ยังไม่เริ่ม</t>
+        </is>
+      </c>
+      <c r="G33" s="4" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+      <c r="H33" s="4" t="inlineStr">
+        <is>
+          <t>ตัวกำหนดว่าจะย้ายแพลตฟอร์มหรือไม่</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="32" customHeight="1">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>Phase 5</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>แผนปิดระบบ</t>
+        </is>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>กำหนดวิธีจัดการยอดที่ไม่มีผู้มาถอนตามระเบียบ</t>
+        </is>
+      </c>
+      <c r="D34" s="5" t="inlineStr">
+        <is>
+          <t>รอกำหนด</t>
+        </is>
+      </c>
+      <c r="E34" s="5" t="inlineStr"/>
+      <c r="F34" s="5" t="inlineStr">
+        <is>
+          <t>ยังไม่เริ่ม</t>
+        </is>
+      </c>
+      <c r="G34" s="5" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+      <c r="H34" s="5" t="inlineStr"/>
+    </row>
+    <row r="35" ht="32" customHeight="1">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Phase 5</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>แผนปิดระบบ</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>วางแผนเก็บข้อมูลถาวร (archive) ให้ค้นย้อนหลังได้</t>
+        </is>
+      </c>
+      <c r="D35" s="4" t="inlineStr">
+        <is>
+          <t>รอกำหนด</t>
+        </is>
+      </c>
+      <c r="E35" s="4" t="inlineStr"/>
+      <c r="F35" s="4" t="inlineStr">
+        <is>
+          <t>ยังไม่เริ่ม</t>
+        </is>
+      </c>
+      <c r="G35" s="4" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+      <c r="H35" s="4" t="inlineStr"/>
+    </row>
+    <row r="36" ht="32" customHeight="1">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Phase 5</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="inlineStr">
+        <is>
+          <t>แผนปิดระบบ</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>กำหนดวิธีให้บริการหากมีผู้มาติดต่อหลังปิดระบบ</t>
+        </is>
+      </c>
+      <c r="D36" s="5" t="inlineStr">
+        <is>
+          <t>รอกำหนด</t>
+        </is>
+      </c>
+      <c r="E36" s="5" t="inlineStr"/>
+      <c r="F36" s="5" t="inlineStr">
+        <is>
+          <t>ยังไม่เริ่ม</t>
+        </is>
+      </c>
+      <c r="G36" s="5" t="inlineStr">
+        <is>
+          <t>ปานกลาง</t>
+        </is>
+      </c>
+      <c r="H36" s="5" t="inlineStr"/>
+    </row>
+    <row r="37" ht="32" customHeight="1">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Phase 5</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>แผนปิดระบบ</t>
+        </is>
+      </c>
+      <c r="C37" s="4" t="inlineStr">
+        <is>
+          <t>ปลดระวางระบบและเพิกถอนสิทธิ์เข้าถึงทั้งหมด</t>
+        </is>
+      </c>
+      <c r="D37" s="4" t="inlineStr">
+        <is>
+          <t>รอกำหนด</t>
+        </is>
+      </c>
+      <c r="E37" s="4" t="inlineStr"/>
+      <c r="F37" s="4" t="inlineStr">
+        <is>
+          <t>ยังไม่เริ่ม</t>
+        </is>
+      </c>
+      <c r="G37" s="4" t="inlineStr">
+        <is>
+          <t>สูง</t>
+        </is>
+      </c>
+      <c r="H37" s="4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>